<commit_message>
Resultados de análisis problema5 (1M iteraciones)
</commit_message>
<xml_diff>
--- a/Nuevos DeepWins/Problem5_SineHighFreq/Res/Comparativa_12_Neuronas.xlsx
+++ b/Nuevos DeepWins/Problem5_SineHighFreq/Res/Comparativa_12_Neuronas.xlsx
@@ -581,42 +581,42 @@
         <v>0.1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.244782</v>
+        <v>0.249328</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1790732846</v>
+        <v>1790732898</v>
       </c>
       <c r="E2" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F2" t="n">
         <v>200000</v>
       </c>
       <c r="G2" t="n">
-        <v>0.555168</v>
+        <v>0.5233989999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>0.596754</v>
+        <v>0.530587</v>
       </c>
       <c r="I2" t="n">
-        <v>0.575211</v>
+        <v>0.526968</v>
       </c>
       <c r="J2" t="n">
-        <v>0.251531</v>
+        <v>0.251055</v>
       </c>
       <c r="K2" t="n">
-        <v>0.6018520000000001</v>
+        <v>0.524887</v>
       </c>
       <c r="L2" t="n">
-        <v>0.580357</v>
+        <v>0.517857</v>
       </c>
       <c r="M2" t="n">
-        <v>0.590909</v>
+        <v>0.521348</v>
       </c>
       <c r="N2" t="n">
         <v>0.2</v>
@@ -652,23 +652,23 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_3.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_5.txt</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z2" t="n">
         <v>12</v>
       </c>
       <c r="AA2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -682,7 +682,7 @@
         <v>0.1</v>
       </c>
       <c r="B3" t="n">
-        <v>0.245622</v>
+        <v>0.245627</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -699,25 +699,25 @@
         <v>200000</v>
       </c>
       <c r="G3" t="n">
-        <v>0.551435</v>
+        <v>0.545349</v>
       </c>
       <c r="H3" t="n">
-        <v>0.575531</v>
+        <v>0.585518</v>
       </c>
       <c r="I3" t="n">
-        <v>0.563225</v>
+        <v>0.56472</v>
       </c>
       <c r="J3" t="n">
-        <v>0.252148</v>
+        <v>0.252193</v>
       </c>
       <c r="K3" t="n">
-        <v>0.5797099999999999</v>
+        <v>0.59292</v>
       </c>
       <c r="L3" t="n">
-        <v>0.535714</v>
+        <v>0.598214</v>
       </c>
       <c r="M3" t="n">
-        <v>0.556845</v>
+        <v>0.5955549999999999</v>
       </c>
       <c r="N3" t="n">
         <v>0.2</v>
@@ -753,7 +753,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_15.txt</t>
+          <t>_2_12_1_1790732846_4.txt</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -783,42 +783,42 @@
         <v>0.1</v>
       </c>
       <c r="B4" t="n">
-        <v>0.249998</v>
+        <v>0.246074</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1790732898</v>
+        <v>1790732846</v>
       </c>
       <c r="E4" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F4" t="n">
         <v>200000</v>
       </c>
       <c r="G4" t="n">
-        <v>0.500625</v>
+        <v>0.519856</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>0.539326</v>
       </c>
       <c r="I4" t="n">
-        <v>0.667222</v>
+        <v>0.529412</v>
       </c>
       <c r="J4" t="n">
-        <v>0.249923</v>
+        <v>0.252421</v>
       </c>
       <c r="K4" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.570093</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>0.544643</v>
       </c>
       <c r="M4" t="n">
-        <v>0.7179489999999999</v>
+        <v>0.557078</v>
       </c>
       <c r="N4" t="n">
         <v>0.2</v>
@@ -854,23 +854,23 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_15.txt</t>
+          <t>_2_12_1_1790732846_5.txt</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z4" t="n">
         <v>12</v>
       </c>
       <c r="AA4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -884,42 +884,42 @@
         <v>0.1</v>
       </c>
       <c r="B5" t="n">
-        <v>0.242524</v>
+        <v>0.249626</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1790732846</v>
+        <v>1790732898</v>
       </c>
       <c r="E5" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F5" t="n">
         <v>200000</v>
       </c>
       <c r="G5" t="n">
-        <v>0.56044</v>
+        <v>0.52551</v>
       </c>
       <c r="H5" t="n">
-        <v>0.573034</v>
+        <v>0.514357</v>
       </c>
       <c r="I5" t="n">
-        <v>0.566667</v>
+        <v>0.5198739999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>0.252608</v>
+        <v>0.250372</v>
       </c>
       <c r="K5" t="n">
-        <v>0.57767</v>
+        <v>0.521127</v>
       </c>
       <c r="L5" t="n">
-        <v>0.53125</v>
+        <v>0.495536</v>
       </c>
       <c r="M5" t="n">
-        <v>0.553488</v>
+        <v>0.508009</v>
       </c>
       <c r="N5" t="n">
         <v>0.2</v>
@@ -955,23 +955,23 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_8.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_1.txt</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z5" t="n">
         <v>12</v>
       </c>
       <c r="AA5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
@@ -985,42 +985,42 @@
         <v>0.1</v>
       </c>
       <c r="B6" t="n">
-        <v>0.249625</v>
+        <v>0.244782</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1790732898</v>
+        <v>1790732846</v>
       </c>
       <c r="E6" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F6" t="n">
         <v>200000</v>
       </c>
       <c r="G6" t="n">
-        <v>0.527389</v>
+        <v>0.555168</v>
       </c>
       <c r="H6" t="n">
-        <v>0.516854</v>
+        <v>0.596754</v>
       </c>
       <c r="I6" t="n">
-        <v>0.522068</v>
+        <v>0.575211</v>
       </c>
       <c r="J6" t="n">
-        <v>0.250261</v>
+        <v>0.251531</v>
       </c>
       <c r="K6" t="n">
-        <v>0.521327</v>
+        <v>0.6018520000000001</v>
       </c>
       <c r="L6" t="n">
-        <v>0.491071</v>
+        <v>0.580357</v>
       </c>
       <c r="M6" t="n">
-        <v>0.5057469999999999</v>
+        <v>0.590909</v>
       </c>
       <c r="N6" t="n">
         <v>0.2</v>
@@ -1056,23 +1056,23 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_4.txt</t>
+          <t>_2_12_1_1790732846_3.txt</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z6" t="n">
         <v>12</v>
       </c>
       <c r="AA6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1086,7 +1086,7 @@
         <v>0.1</v>
       </c>
       <c r="B7" t="n">
-        <v>0.249378</v>
+        <v>0.249777</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1103,25 +1103,25 @@
         <v>200000</v>
       </c>
       <c r="G7" t="n">
-        <v>0.523573</v>
+        <v>0.523457</v>
       </c>
       <c r="H7" t="n">
-        <v>0.526841</v>
+        <v>0.529338</v>
       </c>
       <c r="I7" t="n">
-        <v>0.5252019999999999</v>
+        <v>0.526381</v>
       </c>
       <c r="J7" t="n">
-        <v>0.250515</v>
+        <v>0.249601</v>
       </c>
       <c r="K7" t="n">
-        <v>0.52968</v>
+        <v>0.571429</v>
       </c>
       <c r="L7" t="n">
-        <v>0.517857</v>
+        <v>0.571429</v>
       </c>
       <c r="M7" t="n">
-        <v>0.523702</v>
+        <v>0.571429</v>
       </c>
       <c r="N7" t="n">
         <v>0.2</v>
@@ -1157,7 +1157,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_12.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_13.txt</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
@@ -1187,7 +1187,7 @@
         <v>0.1</v>
       </c>
       <c r="B8" t="n">
-        <v>0.246573</v>
+        <v>0.246153</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1204,25 +1204,25 @@
         <v>200000</v>
       </c>
       <c r="G8" t="n">
-        <v>0.522407</v>
+        <v>0.541717</v>
       </c>
       <c r="H8" t="n">
-        <v>0.509363</v>
+        <v>0.559301</v>
       </c>
       <c r="I8" t="n">
-        <v>0.515803</v>
+        <v>0.550369</v>
       </c>
       <c r="J8" t="n">
-        <v>0.251588</v>
+        <v>0.251996</v>
       </c>
       <c r="K8" t="n">
-        <v>0.571429</v>
+        <v>0.595238</v>
       </c>
       <c r="L8" t="n">
-        <v>0.535714</v>
+        <v>0.558036</v>
       </c>
       <c r="M8" t="n">
-        <v>0.552995</v>
+        <v>0.576037</v>
       </c>
       <c r="N8" t="n">
         <v>0.2</v>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_6.txt</t>
+          <t>_2_12_1_1790732846_1.txt</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
@@ -1288,7 +1288,7 @@
         <v>0.1</v>
       </c>
       <c r="B9" t="n">
-        <v>0.245369</v>
+        <v>0.245842</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1305,25 +1305,25 @@
         <v>200000</v>
       </c>
       <c r="G9" t="n">
-        <v>0.555556</v>
+        <v>0.545139</v>
       </c>
       <c r="H9" t="n">
-        <v>0.630462</v>
+        <v>0.588015</v>
       </c>
       <c r="I9" t="n">
-        <v>0.590643</v>
+        <v>0.565766</v>
       </c>
       <c r="J9" t="n">
-        <v>0.252582</v>
+        <v>0.252034</v>
       </c>
       <c r="K9" t="n">
-        <v>0.589744</v>
+        <v>0.584416</v>
       </c>
       <c r="L9" t="n">
-        <v>0.616071</v>
+        <v>0.602679</v>
       </c>
       <c r="M9" t="n">
-        <v>0.60262</v>
+        <v>0.593407</v>
       </c>
       <c r="N9" t="n">
         <v>0.2</v>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_9.txt</t>
+          <t>_2_12_1_1790732846_18.txt</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
@@ -1389,7 +1389,7 @@
         <v>0.1</v>
       </c>
       <c r="B10" t="n">
-        <v>0.249381</v>
+        <v>0.249625</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1406,25 +1406,25 @@
         <v>200000</v>
       </c>
       <c r="G10" t="n">
-        <v>0.526448</v>
+        <v>0.527389</v>
       </c>
       <c r="H10" t="n">
-        <v>0.521848</v>
+        <v>0.516854</v>
       </c>
       <c r="I10" t="n">
-        <v>0.524138</v>
+        <v>0.522068</v>
       </c>
       <c r="J10" t="n">
-        <v>0.250348</v>
+        <v>0.250261</v>
       </c>
       <c r="K10" t="n">
-        <v>0.532407</v>
+        <v>0.521327</v>
       </c>
       <c r="L10" t="n">
-        <v>0.513393</v>
+        <v>0.491071</v>
       </c>
       <c r="M10" t="n">
-        <v>0.5227270000000001</v>
+        <v>0.5057469999999999</v>
       </c>
       <c r="N10" t="n">
         <v>0.2</v>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_11.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_4.txt</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
@@ -1490,42 +1490,42 @@
         <v>0.1</v>
       </c>
       <c r="B11" t="n">
-        <v>0.245751</v>
+        <v>0.249912</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1790732846</v>
+        <v>1790732898</v>
       </c>
       <c r="E11" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F11" t="n">
         <v>200000</v>
       </c>
       <c r="G11" t="n">
-        <v>0.533898</v>
+        <v>0.514317</v>
       </c>
       <c r="H11" t="n">
-        <v>0.550562</v>
+        <v>0.583021</v>
       </c>
       <c r="I11" t="n">
-        <v>0.542102</v>
+        <v>0.5465179999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>0.25273</v>
+        <v>0.249951</v>
       </c>
       <c r="K11" t="n">
-        <v>0.566502</v>
+        <v>0.542017</v>
       </c>
       <c r="L11" t="n">
-        <v>0.513393</v>
+        <v>0.575893</v>
       </c>
       <c r="M11" t="n">
-        <v>0.538642</v>
+        <v>0.558442</v>
       </c>
       <c r="N11" t="n">
         <v>0.2</v>
@@ -1561,23 +1561,23 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_0.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_9.txt</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z11" t="n">
         <v>12</v>
       </c>
       <c r="AA11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC11" t="inlineStr">
@@ -1591,7 +1591,7 @@
         <v>0.1</v>
       </c>
       <c r="B12" t="n">
-        <v>0.249851</v>
+        <v>0.249512</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1608,25 +1608,25 @@
         <v>200000</v>
       </c>
       <c r="G12" t="n">
-        <v>0.521739</v>
+        <v>0.522424</v>
       </c>
       <c r="H12" t="n">
-        <v>0.539326</v>
+        <v>0.538077</v>
       </c>
       <c r="I12" t="n">
-        <v>0.5303870000000001</v>
+        <v>0.530135</v>
       </c>
       <c r="J12" t="n">
-        <v>0.249248</v>
+        <v>0.249904</v>
       </c>
       <c r="K12" t="n">
-        <v>0.6018520000000001</v>
+        <v>0.540541</v>
       </c>
       <c r="L12" t="n">
-        <v>0.580357</v>
+        <v>0.535714</v>
       </c>
       <c r="M12" t="n">
-        <v>0.590909</v>
+        <v>0.538117</v>
       </c>
       <c r="N12" t="n">
         <v>0.2</v>
@@ -1662,7 +1662,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_10.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_8.txt</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
@@ -1793,7 +1793,7 @@
         <v>0.1</v>
       </c>
       <c r="B14" t="n">
-        <v>0.249711</v>
+        <v>0.249889</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1810,25 +1810,25 @@
         <v>200000</v>
       </c>
       <c r="G14" t="n">
-        <v>0.52754</v>
+        <v>0.515432</v>
       </c>
       <c r="H14" t="n">
-        <v>0.538077</v>
+        <v>0.625468</v>
       </c>
       <c r="I14" t="n">
-        <v>0.532757</v>
+        <v>0.565144</v>
       </c>
       <c r="J14" t="n">
-        <v>0.249938</v>
+        <v>0.250048</v>
       </c>
       <c r="K14" t="n">
-        <v>0.542986</v>
+        <v>0.532567</v>
       </c>
       <c r="L14" t="n">
-        <v>0.535714</v>
+        <v>0.620536</v>
       </c>
       <c r="M14" t="n">
-        <v>0.539326</v>
+        <v>0.573196</v>
       </c>
       <c r="N14" t="n">
         <v>0.2</v>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_16.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_3.txt</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
@@ -1894,42 +1894,42 @@
         <v>0.1</v>
       </c>
       <c r="B15" t="n">
-        <v>0.2498</v>
+        <v>0.244835</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1790732898</v>
+        <v>1790732846</v>
       </c>
       <c r="E15" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F15" t="n">
         <v>200000</v>
       </c>
       <c r="G15" t="n">
-        <v>0.521542</v>
+        <v>0.561424</v>
       </c>
       <c r="H15" t="n">
-        <v>0.574282</v>
+        <v>0.610487</v>
       </c>
       <c r="I15" t="n">
-        <v>0.546643</v>
+        <v>0.584928</v>
       </c>
       <c r="J15" t="n">
-        <v>0.249726</v>
+        <v>0.252084</v>
       </c>
       <c r="K15" t="n">
-        <v>0.570213</v>
+        <v>0.592593</v>
       </c>
       <c r="L15" t="n">
-        <v>0.598214</v>
+        <v>0.571429</v>
       </c>
       <c r="M15" t="n">
-        <v>0.583878</v>
+        <v>0.5818179999999999</v>
       </c>
       <c r="N15" t="n">
         <v>0.2</v>
@@ -1965,23 +1965,23 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_18.txt</t>
+          <t>_2_12_1_1790732846_14.txt</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z15" t="n">
         <v>12</v>
       </c>
       <c r="AA15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
@@ -1995,7 +1995,7 @@
         <v>0.1</v>
       </c>
       <c r="B16" t="n">
-        <v>0.243116</v>
+        <v>0.246333</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -2012,25 +2012,25 @@
         <v>200000</v>
       </c>
       <c r="G16" t="n">
-        <v>0.552204</v>
+        <v>0.5281169999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>0.594257</v>
+        <v>0.539326</v>
       </c>
       <c r="I16" t="n">
-        <v>0.5724590000000001</v>
+        <v>0.533663</v>
       </c>
       <c r="J16" t="n">
-        <v>0.251933</v>
+        <v>0.251814</v>
       </c>
       <c r="K16" t="n">
-        <v>0.572093</v>
+        <v>0.589862</v>
       </c>
       <c r="L16" t="n">
-        <v>0.549107</v>
+        <v>0.571429</v>
       </c>
       <c r="M16" t="n">
-        <v>0.560364</v>
+        <v>0.580499</v>
       </c>
       <c r="N16" t="n">
         <v>0.2</v>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_17.txt</t>
+          <t>_2_12_1_1790732846_7.txt</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
@@ -2096,42 +2096,42 @@
         <v>0.1</v>
       </c>
       <c r="B17" t="n">
-        <v>0.244102</v>
+        <v>0.249251</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1790732846</v>
+        <v>1790732898</v>
       </c>
       <c r="E17" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F17" t="n">
         <v>200000</v>
       </c>
       <c r="G17" t="n">
-        <v>0.557225</v>
+        <v>0.520651</v>
       </c>
       <c r="H17" t="n">
-        <v>0.6017479999999999</v>
+        <v>0.519351</v>
       </c>
       <c r="I17" t="n">
-        <v>0.578631</v>
+        <v>0.52</v>
       </c>
       <c r="J17" t="n">
-        <v>0.251389</v>
+        <v>0.251666</v>
       </c>
       <c r="K17" t="n">
-        <v>0.5944700000000001</v>
+        <v>0.5183489999999999</v>
       </c>
       <c r="L17" t="n">
-        <v>0.575893</v>
+        <v>0.504464</v>
       </c>
       <c r="M17" t="n">
-        <v>0.5850340000000001</v>
+        <v>0.511312</v>
       </c>
       <c r="N17" t="n">
         <v>0.2</v>
@@ -2167,23 +2167,23 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_10.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_2.txt</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z17" t="n">
         <v>12</v>
       </c>
       <c r="AA17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
@@ -2197,7 +2197,7 @@
         <v>0.1</v>
       </c>
       <c r="B18" t="n">
-        <v>0.244835</v>
+        <v>0.244673</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2214,25 +2214,25 @@
         <v>200000</v>
       </c>
       <c r="G18" t="n">
-        <v>0.561424</v>
+        <v>0.5464599999999999</v>
       </c>
       <c r="H18" t="n">
-        <v>0.610487</v>
+        <v>0.616729</v>
       </c>
       <c r="I18" t="n">
-        <v>0.584928</v>
+        <v>0.579472</v>
       </c>
       <c r="J18" t="n">
-        <v>0.252084</v>
+        <v>0.251644</v>
       </c>
       <c r="K18" t="n">
-        <v>0.592593</v>
+        <v>0.590909</v>
       </c>
       <c r="L18" t="n">
-        <v>0.571429</v>
+        <v>0.580357</v>
       </c>
       <c r="M18" t="n">
-        <v>0.5818179999999999</v>
+        <v>0.5855860000000001</v>
       </c>
       <c r="N18" t="n">
         <v>0.2</v>
@@ -2268,7 +2268,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_14.txt</t>
+          <t>_2_12_1_1790732846_13.txt</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
@@ -2298,7 +2298,7 @@
         <v>0.1</v>
       </c>
       <c r="B19" t="n">
-        <v>0.245627</v>
+        <v>0.244102</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2315,25 +2315,25 @@
         <v>200000</v>
       </c>
       <c r="G19" t="n">
-        <v>0.545349</v>
+        <v>0.557225</v>
       </c>
       <c r="H19" t="n">
-        <v>0.585518</v>
+        <v>0.6017479999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>0.56472</v>
+        <v>0.578631</v>
       </c>
       <c r="J19" t="n">
-        <v>0.252193</v>
+        <v>0.251389</v>
       </c>
       <c r="K19" t="n">
-        <v>0.59292</v>
+        <v>0.5944700000000001</v>
       </c>
       <c r="L19" t="n">
-        <v>0.598214</v>
+        <v>0.575893</v>
       </c>
       <c r="M19" t="n">
-        <v>0.5955549999999999</v>
+        <v>0.5850340000000001</v>
       </c>
       <c r="N19" t="n">
         <v>0.2</v>
@@ -2369,7 +2369,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_4.txt</t>
+          <t>_2_12_1_1790732846_10.txt</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
@@ -2399,42 +2399,42 @@
         <v>0.1</v>
       </c>
       <c r="B20" t="n">
-        <v>0.249328</v>
+        <v>0.243617</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1790732898</v>
+        <v>1790732846</v>
       </c>
       <c r="E20" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F20" t="n">
         <v>200000</v>
       </c>
       <c r="G20" t="n">
-        <v>0.5233989999999999</v>
+        <v>0.549234</v>
       </c>
       <c r="H20" t="n">
-        <v>0.530587</v>
+        <v>0.626717</v>
       </c>
       <c r="I20" t="n">
-        <v>0.526968</v>
+        <v>0.585423</v>
       </c>
       <c r="J20" t="n">
-        <v>0.251055</v>
+        <v>0.251376</v>
       </c>
       <c r="K20" t="n">
-        <v>0.524887</v>
+        <v>0.587983</v>
       </c>
       <c r="L20" t="n">
-        <v>0.517857</v>
+        <v>0.611607</v>
       </c>
       <c r="M20" t="n">
-        <v>0.521348</v>
+        <v>0.599562</v>
       </c>
       <c r="N20" t="n">
         <v>0.2</v>
@@ -2470,23 +2470,23 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_5.txt</t>
+          <t>_2_12_1_1790732846_19.txt</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z20" t="n">
         <v>12</v>
       </c>
       <c r="AA20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC20" t="inlineStr">
@@ -2500,42 +2500,42 @@
         <v>0.1</v>
       </c>
       <c r="B21" t="n">
-        <v>0.245049</v>
+        <v>0.249998</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1790732846</v>
+        <v>1790732898</v>
       </c>
       <c r="E21" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F21" t="n">
         <v>200000</v>
       </c>
       <c r="G21" t="n">
-        <v>0.559719</v>
+        <v>0.500625</v>
       </c>
       <c r="H21" t="n">
-        <v>0.596754</v>
+        <v>1</v>
       </c>
       <c r="I21" t="n">
-        <v>0.577644</v>
+        <v>0.667222</v>
       </c>
       <c r="J21" t="n">
-        <v>0.252427</v>
+        <v>0.249923</v>
       </c>
       <c r="K21" t="n">
-        <v>0.593607</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="L21" t="n">
-        <v>0.580357</v>
+        <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>0.586907</v>
+        <v>0.7179489999999999</v>
       </c>
       <c r="N21" t="n">
         <v>0.2</v>
@@ -2571,23 +2571,23 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_12.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_15.txt</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z21" t="n">
         <v>12</v>
       </c>
       <c r="AA21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC21" t="inlineStr">
@@ -2601,7 +2601,7 @@
         <v>0.1</v>
       </c>
       <c r="B22" t="n">
-        <v>0.249913</v>
+        <v>0.249969</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -2618,25 +2618,25 @@
         <v>200000</v>
       </c>
       <c r="G22" t="n">
-        <v>0.520085</v>
+        <v>0.50506</v>
       </c>
       <c r="H22" t="n">
-        <v>0.614232</v>
+        <v>0.685393</v>
       </c>
       <c r="I22" t="n">
-        <v>0.5632509999999999</v>
+        <v>0.581568</v>
       </c>
       <c r="J22" t="n">
-        <v>0.249677</v>
+        <v>0.250024</v>
       </c>
       <c r="K22" t="n">
-        <v>0.602459</v>
+        <v>0.5161289999999999</v>
       </c>
       <c r="L22" t="n">
-        <v>0.65625</v>
+        <v>0.642857</v>
       </c>
       <c r="M22" t="n">
-        <v>0.628205</v>
+        <v>0.572565</v>
       </c>
       <c r="N22" t="n">
         <v>0.2</v>
@@ -2672,7 +2672,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_14.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_19.txt</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
@@ -2702,7 +2702,7 @@
         <v>0.1</v>
       </c>
       <c r="B23" t="n">
-        <v>0.249293</v>
+        <v>0.249851</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2719,25 +2719,25 @@
         <v>200000</v>
       </c>
       <c r="G23" t="n">
-        <v>0.52859</v>
+        <v>0.521739</v>
       </c>
       <c r="H23" t="n">
-        <v>0.519351</v>
+        <v>0.539326</v>
       </c>
       <c r="I23" t="n">
-        <v>0.523929</v>
+        <v>0.5303870000000001</v>
       </c>
       <c r="J23" t="n">
-        <v>0.250999</v>
+        <v>0.249248</v>
       </c>
       <c r="K23" t="n">
-        <v>0.532407</v>
+        <v>0.6018520000000001</v>
       </c>
       <c r="L23" t="n">
-        <v>0.513393</v>
+        <v>0.580357</v>
       </c>
       <c r="M23" t="n">
-        <v>0.5227270000000001</v>
+        <v>0.590909</v>
       </c>
       <c r="N23" t="n">
         <v>0.2</v>
@@ -2773,7 +2773,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_0.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_10.txt</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
@@ -2803,7 +2803,7 @@
         <v>0.1</v>
       </c>
       <c r="B24" t="n">
-        <v>0.249806</v>
+        <v>0.249156</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2820,25 +2820,25 @@
         <v>200000</v>
       </c>
       <c r="G24" t="n">
-        <v>0.5172</v>
+        <v>0.521472</v>
       </c>
       <c r="H24" t="n">
-        <v>0.54432</v>
+        <v>0.530587</v>
       </c>
       <c r="I24" t="n">
-        <v>0.5304140000000001</v>
+        <v>0.52599</v>
       </c>
       <c r="J24" t="n">
-        <v>0.250343</v>
+        <v>0.2508</v>
       </c>
       <c r="K24" t="n">
-        <v>0.526316</v>
+        <v>0.529412</v>
       </c>
       <c r="L24" t="n">
-        <v>0.535714</v>
+        <v>0.522321</v>
       </c>
       <c r="M24" t="n">
-        <v>0.530973</v>
+        <v>0.5258429999999999</v>
       </c>
       <c r="N24" t="n">
         <v>0.2</v>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_17.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_7.txt</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
@@ -2904,42 +2904,42 @@
         <v>0.1</v>
       </c>
       <c r="B25" t="n">
-        <v>0.249912</v>
+        <v>0.246019</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>1790732898</v>
+        <v>1790732846</v>
       </c>
       <c r="E25" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F25" t="n">
         <v>200000</v>
       </c>
       <c r="G25" t="n">
-        <v>0.514317</v>
+        <v>0.539863</v>
       </c>
       <c r="H25" t="n">
-        <v>0.583021</v>
+        <v>0.59176</v>
       </c>
       <c r="I25" t="n">
-        <v>0.5465179999999999</v>
+        <v>0.564622</v>
       </c>
       <c r="J25" t="n">
-        <v>0.249951</v>
+        <v>0.2511</v>
       </c>
       <c r="K25" t="n">
-        <v>0.542017</v>
+        <v>0.592105</v>
       </c>
       <c r="L25" t="n">
-        <v>0.575893</v>
+        <v>0.602679</v>
       </c>
       <c r="M25" t="n">
-        <v>0.558442</v>
+        <v>0.597345</v>
       </c>
       <c r="N25" t="n">
         <v>0.2</v>
@@ -2975,23 +2975,23 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_9.txt</t>
+          <t>_2_12_1_1790732846_2.txt</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z25" t="n">
         <v>12</v>
       </c>
       <c r="AA25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB25" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC25" t="inlineStr">
@@ -3005,42 +3005,42 @@
         <v>0.1</v>
       </c>
       <c r="B26" t="n">
-        <v>0.246019</v>
+        <v>0.2498</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1790732846</v>
+        <v>1790732898</v>
       </c>
       <c r="E26" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F26" t="n">
         <v>200000</v>
       </c>
       <c r="G26" t="n">
-        <v>0.539863</v>
+        <v>0.521542</v>
       </c>
       <c r="H26" t="n">
-        <v>0.59176</v>
+        <v>0.574282</v>
       </c>
       <c r="I26" t="n">
-        <v>0.564622</v>
+        <v>0.546643</v>
       </c>
       <c r="J26" t="n">
-        <v>0.2511</v>
+        <v>0.249726</v>
       </c>
       <c r="K26" t="n">
-        <v>0.592105</v>
+        <v>0.570213</v>
       </c>
       <c r="L26" t="n">
-        <v>0.602679</v>
+        <v>0.598214</v>
       </c>
       <c r="M26" t="n">
-        <v>0.597345</v>
+        <v>0.583878</v>
       </c>
       <c r="N26" t="n">
         <v>0.2</v>
@@ -3076,23 +3076,23 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_2.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_18.txt</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z26" t="n">
         <v>12</v>
       </c>
       <c r="AA26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB26" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC26" t="inlineStr">
@@ -3106,42 +3106,42 @@
         <v>0.1</v>
       </c>
       <c r="B27" t="n">
-        <v>0.246153</v>
+        <v>0.249293</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1790732846</v>
+        <v>1790732898</v>
       </c>
       <c r="E27" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F27" t="n">
         <v>200000</v>
       </c>
       <c r="G27" t="n">
-        <v>0.541717</v>
+        <v>0.52859</v>
       </c>
       <c r="H27" t="n">
-        <v>0.559301</v>
+        <v>0.519351</v>
       </c>
       <c r="I27" t="n">
-        <v>0.550369</v>
+        <v>0.523929</v>
       </c>
       <c r="J27" t="n">
-        <v>0.251996</v>
+        <v>0.250999</v>
       </c>
       <c r="K27" t="n">
-        <v>0.595238</v>
+        <v>0.532407</v>
       </c>
       <c r="L27" t="n">
-        <v>0.558036</v>
+        <v>0.513393</v>
       </c>
       <c r="M27" t="n">
-        <v>0.576037</v>
+        <v>0.5227270000000001</v>
       </c>
       <c r="N27" t="n">
         <v>0.2</v>
@@ -3177,23 +3177,23 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_1.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_0.txt</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z27" t="n">
         <v>12</v>
       </c>
       <c r="AA27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB27" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC27" t="inlineStr">
@@ -3207,42 +3207,42 @@
         <v>0.1</v>
       </c>
       <c r="B28" t="n">
-        <v>0.249372</v>
+        <v>0.245049</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1790732898</v>
+        <v>1790732846</v>
       </c>
       <c r="E28" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F28" t="n">
         <v>200000</v>
       </c>
       <c r="G28" t="n">
-        <v>0.5264450000000001</v>
+        <v>0.559719</v>
       </c>
       <c r="H28" t="n">
-        <v>0.534332</v>
+        <v>0.596754</v>
       </c>
       <c r="I28" t="n">
-        <v>0.530359</v>
+        <v>0.577644</v>
       </c>
       <c r="J28" t="n">
-        <v>0.25011</v>
+        <v>0.252427</v>
       </c>
       <c r="K28" t="n">
-        <v>0.534247</v>
+        <v>0.593607</v>
       </c>
       <c r="L28" t="n">
-        <v>0.522321</v>
+        <v>0.580357</v>
       </c>
       <c r="M28" t="n">
-        <v>0.528217</v>
+        <v>0.586907</v>
       </c>
       <c r="N28" t="n">
         <v>0.2</v>
@@ -3278,23 +3278,23 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_6.txt</t>
+          <t>_2_12_1_1790732846_12.txt</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z28" t="n">
         <v>12</v>
       </c>
       <c r="AA28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB28" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC28" t="inlineStr">
@@ -3308,7 +3308,7 @@
         <v>0.1</v>
       </c>
       <c r="B29" t="n">
-        <v>0.243617</v>
+        <v>0.242524</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3325,25 +3325,25 @@
         <v>200000</v>
       </c>
       <c r="G29" t="n">
-        <v>0.549234</v>
+        <v>0.56044</v>
       </c>
       <c r="H29" t="n">
-        <v>0.626717</v>
+        <v>0.573034</v>
       </c>
       <c r="I29" t="n">
-        <v>0.585423</v>
+        <v>0.566667</v>
       </c>
       <c r="J29" t="n">
-        <v>0.251376</v>
+        <v>0.252608</v>
       </c>
       <c r="K29" t="n">
-        <v>0.587983</v>
+        <v>0.57767</v>
       </c>
       <c r="L29" t="n">
-        <v>0.611607</v>
+        <v>0.53125</v>
       </c>
       <c r="M29" t="n">
-        <v>0.599562</v>
+        <v>0.553488</v>
       </c>
       <c r="N29" t="n">
         <v>0.2</v>
@@ -3379,7 +3379,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_19.txt</t>
+          <t>_2_12_1_1790732846_8.txt</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
@@ -3409,7 +3409,7 @@
         <v>0.1</v>
       </c>
       <c r="B30" t="n">
-        <v>0.249889</v>
+        <v>0.249378</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -3426,25 +3426,25 @@
         <v>200000</v>
       </c>
       <c r="G30" t="n">
-        <v>0.515432</v>
+        <v>0.523573</v>
       </c>
       <c r="H30" t="n">
-        <v>0.625468</v>
+        <v>0.526841</v>
       </c>
       <c r="I30" t="n">
-        <v>0.565144</v>
+        <v>0.5252019999999999</v>
       </c>
       <c r="J30" t="n">
-        <v>0.250048</v>
+        <v>0.250515</v>
       </c>
       <c r="K30" t="n">
-        <v>0.532567</v>
+        <v>0.52968</v>
       </c>
       <c r="L30" t="n">
-        <v>0.620536</v>
+        <v>0.517857</v>
       </c>
       <c r="M30" t="n">
-        <v>0.573196</v>
+        <v>0.523702</v>
       </c>
       <c r="N30" t="n">
         <v>0.2</v>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_3.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_12.txt</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
@@ -3510,7 +3510,7 @@
         <v>0.1</v>
       </c>
       <c r="B31" t="n">
-        <v>0.246333</v>
+        <v>0.245751</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3527,25 +3527,25 @@
         <v>200000</v>
       </c>
       <c r="G31" t="n">
-        <v>0.5281169999999999</v>
+        <v>0.533898</v>
       </c>
       <c r="H31" t="n">
-        <v>0.539326</v>
+        <v>0.550562</v>
       </c>
       <c r="I31" t="n">
-        <v>0.533663</v>
+        <v>0.542102</v>
       </c>
       <c r="J31" t="n">
-        <v>0.251814</v>
+        <v>0.25273</v>
       </c>
       <c r="K31" t="n">
-        <v>0.589862</v>
+        <v>0.566502</v>
       </c>
       <c r="L31" t="n">
-        <v>0.571429</v>
+        <v>0.513393</v>
       </c>
       <c r="M31" t="n">
-        <v>0.580499</v>
+        <v>0.538642</v>
       </c>
       <c r="N31" t="n">
         <v>0.2</v>
@@ -3581,7 +3581,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_7.txt</t>
+          <t>_2_12_1_1790732846_0.txt</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
@@ -3611,42 +3611,42 @@
         <v>0.1</v>
       </c>
       <c r="B32" t="n">
-        <v>0.245842</v>
+        <v>0.249381</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1790732846</v>
+        <v>1790732898</v>
       </c>
       <c r="E32" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F32" t="n">
         <v>200000</v>
       </c>
       <c r="G32" t="n">
-        <v>0.545139</v>
+        <v>0.526448</v>
       </c>
       <c r="H32" t="n">
-        <v>0.588015</v>
+        <v>0.521848</v>
       </c>
       <c r="I32" t="n">
-        <v>0.565766</v>
+        <v>0.524138</v>
       </c>
       <c r="J32" t="n">
-        <v>0.252034</v>
+        <v>0.250348</v>
       </c>
       <c r="K32" t="n">
-        <v>0.584416</v>
+        <v>0.532407</v>
       </c>
       <c r="L32" t="n">
-        <v>0.602679</v>
+        <v>0.513393</v>
       </c>
       <c r="M32" t="n">
-        <v>0.593407</v>
+        <v>0.5227270000000001</v>
       </c>
       <c r="N32" t="n">
         <v>0.2</v>
@@ -3682,23 +3682,23 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_18.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_11.txt</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z32" t="n">
         <v>12</v>
       </c>
       <c r="AA32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC32" t="inlineStr">
@@ -3712,42 +3712,42 @@
         <v>0.1</v>
       </c>
       <c r="B33" t="n">
-        <v>0.249512</v>
+        <v>0.245622</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1790732898</v>
+        <v>1790732846</v>
       </c>
       <c r="E33" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F33" t="n">
         <v>200000</v>
       </c>
       <c r="G33" t="n">
-        <v>0.522424</v>
+        <v>0.551435</v>
       </c>
       <c r="H33" t="n">
-        <v>0.538077</v>
+        <v>0.575531</v>
       </c>
       <c r="I33" t="n">
-        <v>0.530135</v>
+        <v>0.563225</v>
       </c>
       <c r="J33" t="n">
-        <v>0.249904</v>
+        <v>0.252148</v>
       </c>
       <c r="K33" t="n">
-        <v>0.540541</v>
+        <v>0.5797099999999999</v>
       </c>
       <c r="L33" t="n">
         <v>0.535714</v>
       </c>
       <c r="M33" t="n">
-        <v>0.538117</v>
+        <v>0.556845</v>
       </c>
       <c r="N33" t="n">
         <v>0.2</v>
@@ -3783,23 +3783,23 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_8.txt</t>
+          <t>_2_12_1_1790732846_15.txt</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z33" t="n">
         <v>12</v>
       </c>
       <c r="AA33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB33" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC33" t="inlineStr">
@@ -3813,7 +3813,7 @@
         <v>0.1</v>
       </c>
       <c r="B34" t="n">
-        <v>0.249156</v>
+        <v>0.249913</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -3830,25 +3830,25 @@
         <v>200000</v>
       </c>
       <c r="G34" t="n">
-        <v>0.521472</v>
+        <v>0.520085</v>
       </c>
       <c r="H34" t="n">
-        <v>0.530587</v>
+        <v>0.614232</v>
       </c>
       <c r="I34" t="n">
-        <v>0.52599</v>
+        <v>0.5632509999999999</v>
       </c>
       <c r="J34" t="n">
-        <v>0.2508</v>
+        <v>0.249677</v>
       </c>
       <c r="K34" t="n">
-        <v>0.529412</v>
+        <v>0.602459</v>
       </c>
       <c r="L34" t="n">
-        <v>0.522321</v>
+        <v>0.65625</v>
       </c>
       <c r="M34" t="n">
-        <v>0.5258429999999999</v>
+        <v>0.628205</v>
       </c>
       <c r="N34" t="n">
         <v>0.2</v>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_7.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_14.txt</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
@@ -3914,42 +3914,42 @@
         <v>0.1</v>
       </c>
       <c r="B35" t="n">
-        <v>0.249969</v>
+        <v>0.243116</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1790732898</v>
+        <v>1790732846</v>
       </c>
       <c r="E35" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F35" t="n">
         <v>200000</v>
       </c>
       <c r="G35" t="n">
-        <v>0.50506</v>
+        <v>0.552204</v>
       </c>
       <c r="H35" t="n">
-        <v>0.685393</v>
+        <v>0.594257</v>
       </c>
       <c r="I35" t="n">
-        <v>0.581568</v>
+        <v>0.5724590000000001</v>
       </c>
       <c r="J35" t="n">
-        <v>0.250024</v>
+        <v>0.251933</v>
       </c>
       <c r="K35" t="n">
-        <v>0.5161289999999999</v>
+        <v>0.572093</v>
       </c>
       <c r="L35" t="n">
-        <v>0.642857</v>
+        <v>0.549107</v>
       </c>
       <c r="M35" t="n">
-        <v>0.572565</v>
+        <v>0.560364</v>
       </c>
       <c r="N35" t="n">
         <v>0.2</v>
@@ -3985,23 +3985,23 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_19.txt</t>
+          <t>_2_12_1_1790732846_17.txt</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z35" t="n">
         <v>12</v>
       </c>
       <c r="AA35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB35" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC35" t="inlineStr">
@@ -4015,7 +4015,7 @@
         <v>0.1</v>
       </c>
       <c r="B36" t="n">
-        <v>0.245823</v>
+        <v>0.245369</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -4032,25 +4032,25 @@
         <v>200000</v>
       </c>
       <c r="G36" t="n">
-        <v>0.550996</v>
+        <v>0.555556</v>
       </c>
       <c r="H36" t="n">
-        <v>0.586767</v>
+        <v>0.630462</v>
       </c>
       <c r="I36" t="n">
-        <v>0.568319</v>
+        <v>0.590643</v>
       </c>
       <c r="J36" t="n">
-        <v>0.251529</v>
+        <v>0.252582</v>
       </c>
       <c r="K36" t="n">
-        <v>0.582569</v>
+        <v>0.589744</v>
       </c>
       <c r="L36" t="n">
-        <v>0.566964</v>
+        <v>0.616071</v>
       </c>
       <c r="M36" t="n">
-        <v>0.574661</v>
+        <v>0.60262</v>
       </c>
       <c r="N36" t="n">
         <v>0.2</v>
@@ -4086,7 +4086,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_16.txt</t>
+          <t>_2_12_1_1790732846_9.txt</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
@@ -4116,42 +4116,42 @@
         <v>0.1</v>
       </c>
       <c r="B37" t="n">
-        <v>0.249251</v>
+        <v>0.246573</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_</t>
+          <t>_2_12_1_</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1790732898</v>
+        <v>1790732846</v>
       </c>
       <c r="E37" t="n">
-        <v>171</v>
+        <v>52</v>
       </c>
       <c r="F37" t="n">
         <v>200000</v>
       </c>
       <c r="G37" t="n">
-        <v>0.520651</v>
+        <v>0.522407</v>
       </c>
       <c r="H37" t="n">
-        <v>0.519351</v>
+        <v>0.509363</v>
       </c>
       <c r="I37" t="n">
-        <v>0.52</v>
+        <v>0.515803</v>
       </c>
       <c r="J37" t="n">
-        <v>0.251666</v>
+        <v>0.251588</v>
       </c>
       <c r="K37" t="n">
-        <v>0.5183489999999999</v>
+        <v>0.571429</v>
       </c>
       <c r="L37" t="n">
-        <v>0.504464</v>
+        <v>0.535714</v>
       </c>
       <c r="M37" t="n">
-        <v>0.511312</v>
+        <v>0.552995</v>
       </c>
       <c r="N37" t="n">
         <v>0.2</v>
@@ -4187,23 +4187,23 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_2.txt</t>
+          <t>_2_12_1_1790732846_6.txt</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t>[3, 3, 3, 3]</t>
+          <t>[12]</t>
         </is>
       </c>
       <c r="Z37" t="n">
         <v>12</v>
       </c>
       <c r="AA37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>Profunda</t>
+          <t>Angosta</t>
         </is>
       </c>
       <c r="AC37" t="inlineStr">
@@ -4217,42 +4217,42 @@
         <v>0.1</v>
       </c>
       <c r="B38" t="n">
-        <v>0.246074</v>
+        <v>0.249711</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>_2_12_1_</t>
+          <t>_2_3_3_3_3_1_</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1790732846</v>
+        <v>1790732898</v>
       </c>
       <c r="E38" t="n">
-        <v>52</v>
+        <v>171</v>
       </c>
       <c r="F38" t="n">
         <v>200000</v>
       </c>
       <c r="G38" t="n">
-        <v>0.519856</v>
+        <v>0.52754</v>
       </c>
       <c r="H38" t="n">
+        <v>0.538077</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.532757</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0.249938</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0.542986</v>
+      </c>
+      <c r="L38" t="n">
+        <v>0.535714</v>
+      </c>
+      <c r="M38" t="n">
         <v>0.539326</v>
-      </c>
-      <c r="I38" t="n">
-        <v>0.529412</v>
-      </c>
-      <c r="J38" t="n">
-        <v>0.252421</v>
-      </c>
-      <c r="K38" t="n">
-        <v>0.570093</v>
-      </c>
-      <c r="L38" t="n">
-        <v>0.544643</v>
-      </c>
-      <c r="M38" t="n">
-        <v>0.557078</v>
       </c>
       <c r="N38" t="n">
         <v>0.2</v>
@@ -4288,23 +4288,23 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_5.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_16.txt</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[3, 3, 3, 3]</t>
         </is>
       </c>
       <c r="Z38" t="n">
         <v>12</v>
       </c>
       <c r="AA38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>Angosta</t>
+          <t>Profunda</t>
         </is>
       </c>
       <c r="AC38" t="inlineStr">
@@ -4318,7 +4318,7 @@
         <v>0.1</v>
       </c>
       <c r="B39" t="n">
-        <v>0.249777</v>
+        <v>0.249806</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -4335,25 +4335,25 @@
         <v>200000</v>
       </c>
       <c r="G39" t="n">
-        <v>0.523457</v>
+        <v>0.5172</v>
       </c>
       <c r="H39" t="n">
-        <v>0.529338</v>
+        <v>0.54432</v>
       </c>
       <c r="I39" t="n">
-        <v>0.526381</v>
+        <v>0.5304140000000001</v>
       </c>
       <c r="J39" t="n">
-        <v>0.249601</v>
+        <v>0.250343</v>
       </c>
       <c r="K39" t="n">
-        <v>0.571429</v>
+        <v>0.526316</v>
       </c>
       <c r="L39" t="n">
-        <v>0.571429</v>
+        <v>0.535714</v>
       </c>
       <c r="M39" t="n">
-        <v>0.571429</v>
+        <v>0.530973</v>
       </c>
       <c r="N39" t="n">
         <v>0.2</v>
@@ -4389,7 +4389,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_13.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_17.txt</t>
         </is>
       </c>
       <c r="Y39" t="inlineStr">
@@ -4419,7 +4419,7 @@
         <v>0.1</v>
       </c>
       <c r="B40" t="n">
-        <v>0.249626</v>
+        <v>0.249372</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -4436,25 +4436,25 @@
         <v>200000</v>
       </c>
       <c r="G40" t="n">
-        <v>0.52551</v>
+        <v>0.5264450000000001</v>
       </c>
       <c r="H40" t="n">
-        <v>0.514357</v>
+        <v>0.534332</v>
       </c>
       <c r="I40" t="n">
-        <v>0.5198739999999999</v>
+        <v>0.530359</v>
       </c>
       <c r="J40" t="n">
-        <v>0.250372</v>
+        <v>0.25011</v>
       </c>
       <c r="K40" t="n">
-        <v>0.521127</v>
+        <v>0.534247</v>
       </c>
       <c r="L40" t="n">
-        <v>0.495536</v>
+        <v>0.522321</v>
       </c>
       <c r="M40" t="n">
-        <v>0.508009</v>
+        <v>0.528217</v>
       </c>
       <c r="N40" t="n">
         <v>0.2</v>
@@ -4490,7 +4490,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>_2_3_3_3_3_1_1790732898_1.txt</t>
+          <t>_2_3_3_3_3_1_1790732898_6.txt</t>
         </is>
       </c>
       <c r="Y40" t="inlineStr">
@@ -4520,7 +4520,7 @@
         <v>0.1</v>
       </c>
       <c r="B41" t="n">
-        <v>0.244673</v>
+        <v>0.245823</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -4537,25 +4537,25 @@
         <v>200000</v>
       </c>
       <c r="G41" t="n">
-        <v>0.5464599999999999</v>
+        <v>0.550996</v>
       </c>
       <c r="H41" t="n">
-        <v>0.616729</v>
+        <v>0.586767</v>
       </c>
       <c r="I41" t="n">
-        <v>0.579472</v>
+        <v>0.568319</v>
       </c>
       <c r="J41" t="n">
-        <v>0.251644</v>
+        <v>0.251529</v>
       </c>
       <c r="K41" t="n">
-        <v>0.590909</v>
+        <v>0.582569</v>
       </c>
       <c r="L41" t="n">
-        <v>0.580357</v>
+        <v>0.566964</v>
       </c>
       <c r="M41" t="n">
-        <v>0.5855860000000001</v>
+        <v>0.574661</v>
       </c>
       <c r="N41" t="n">
         <v>0.2</v>
@@ -4591,7 +4591,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>_2_12_1_1790732846_13.txt</t>
+          <t>_2_12_1_1790732846_16.txt</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
@@ -4682,7 +4682,7 @@
         <v>0.5770717000000001</v>
       </c>
       <c r="C2" t="n">
-        <v>0.01830860264322127</v>
+        <v>0.01830860264322125</v>
       </c>
       <c r="D2" t="n">
         <v>0.60262</v>
@@ -4710,7 +4710,7 @@
         <v>0.55373105</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0504386844995981</v>
+        <v>0.05043868449959812</v>
       </c>
       <c r="D3" t="n">
         <v>0.7179489999999999</v>

</xml_diff>